<commit_message>
auto: update flight data
</commit_message>
<xml_diff>
--- a/flight_data/live_flights.xlsx
+++ b/flight_data/live_flights.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,830 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>OV761</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Salam Air</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0025</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OV421</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Salam Air</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sylhet</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sylhet</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0045</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OV401</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salam Air</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Chattogram</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Chattogram</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0115</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0151</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WY685</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Oman Air</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Riyadh</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Riyadh</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0145</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WY849</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Oman Air</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0150</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BS322</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0200</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TK775</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Turkish Airlines</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Istanbul</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Istanbul</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0210</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WY251</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Oman Air</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WY225</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Oman Air</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0225</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WY211</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Oman Air</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0225</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6E1274</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6E</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0250</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IX442</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0250</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WY265</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Oman Air</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6E1272</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>6E</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OV513</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Salam Air</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Karachi</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Karachi</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0315</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>IX236</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>24SEP</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0015</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Departed</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-09-24 00:01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>